<commit_message>
updated dependencies, adapted input file handling and outdir creation, added test cases and updated README
</commit_message>
<xml_diff>
--- a/assets/data/test_table_3.xlsx
+++ b/assets/data/test_table_3.xlsx
@@ -5,11 +5,11 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Tabelle2" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="Tabelle1" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="Tabelle2" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Tabelle1" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -23,16 +23,16 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="28">
   <si>
-    <t xml:space="preserve">Test1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test4</t>
+    <t xml:space="preserve">col_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">col_2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">col_3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">col_4</t>
   </si>
   <si>
     <t xml:space="preserve">asdf</t>
@@ -184,7 +184,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -200,8 +200,114 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -561,7 +667,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;A</oddHeader>
     <oddFooter>&amp;CSeite &amp;P</oddFooter>
@@ -570,7 +676,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -852,7 +958,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;A</oddHeader>
     <oddFooter>&amp;CSeite &amp;P</oddFooter>

</xml_diff>